<commit_message>
Disable conditional formatting in seq_info.xlsx
</commit_message>
<xml_diff>
--- a/sample_data/a_Stx-phages/seq_info.xlsx
+++ b/sample_data/a_Stx-phages/seq_info.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okuno/Documents/work/2025_lyla2/github/sample_data/a_Stx-phages/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okuno/tools/lyla-plot/for_bioconda/a-liner/sample_data/a_Stx-phages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DF0721-9D65-3A4A-B3D4-03EEC9C1F778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D603D8A-0C77-6443-A338-1992F74C3EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-65060" yWindow="2820" windowWidth="28400" windowHeight="18360" xr2:uid="{9A43F9C3-30CB-2542-B04D-2F0B62A57818}"/>
   </bookViews>
@@ -204,7 +204,7 @@
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="7">
     <dxf>
       <font>
         <color rgb="FFFF40FF"/>
@@ -218,6 +218,36 @@
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF40FF"/>
       </font>
       <fill>
         <patternFill>
@@ -699,20 +729,15 @@
   </sortState>
   <phoneticPr fontId="1"/>
   <conditionalFormatting sqref="A2:A7 A10:A1048576">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="greaterThanOrEqual">
       <formula>COUNTA($A$2:$A$1048576)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:F7 A10:F1048576">
-    <cfRule type="expression" dxfId="1" priority="9">
-      <formula>COUNTA($A$2:$A$1048576)*(COUNTA($A$2:$A$1048576)-1)/2-SUM($A$2:$A$1048576)&lt;&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E2:E7 E10:E1048576">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>NOT(OR((E2 = "+"), (E2 = "-")))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>